<commit_message>
Update Excel: weekly swim technique themes with full session details
</commit_message>
<xml_diff>
--- a/plan/training_plan_12weeks.xlsx
+++ b/plan/training_plan_12weeks.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="12周铁三训练计划" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="游泳技术路线" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'12周铁三训练计划'!$A$1:$J$14</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'12周铁三训练计划'!$A$1:$I$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,9 +36,14 @@
     </font>
     <font>
       <name val="微软雅黑"/>
+      <color rgb="001A5276"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="9"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <name val="微软雅黑"/>
@@ -60,8 +66,26 @@
       <color rgb="00555555"/>
       <sz val="7.5"/>
     </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -70,7 +94,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002C3E50"/>
+        <fgColor rgb="001A5276"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EEF8"/>
       </patternFill>
     </fill>
     <fill>
@@ -86,6 +115,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EBF5FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F8F5"/>
       </patternFill>
     </fill>
     <fill>
@@ -128,6 +162,16 @@
         <fgColor rgb="00F0F0F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0FBF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8F8F8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -139,16 +183,16 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="00888888"/>
+        <color rgb="00666666"/>
       </left>
       <right style="medium">
-        <color rgb="00888888"/>
+        <color rgb="00666666"/>
       </right>
       <top style="medium">
-        <color rgb="00888888"/>
+        <color rgb="00666666"/>
       </top>
       <bottom style="medium">
-        <color rgb="00888888"/>
+        <color rgb="00666666"/>
       </bottom>
     </border>
     <border>
@@ -169,49 +213,70 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -578,109 +643,118 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Zikun Sprint Triathlon 12-Week Training Plan  |  Race: 2026-05-30  |  HRmax: 186 bpm  |  Z2:114-132  Z3:133-150  Z4:151-165  Z5:&gt;165</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="42" customHeight="1">
+          <t>Zikun Sprint Triathlon · 12-Week Training Plan · Race: 2026-05-30 · HRmax 186bpm · Z2:114-132 · Z3:133-150 · Z4:151-165</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>周次</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+          <t>🏊 游泳技术路线：Wk1–2 单臂划水 → Wk3–4 追手/滑翔 → Wk5–6 双侧呼吸 → Wk7–8 打腿节奏 → Wk9–10 整合配速 → Wk11 减量 → Wk12 激活</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>周次
+日期</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>阶段</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>周一
 Mon
-休息</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+💤REST</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>周二
 Tue
-跑步(间歇)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+🏃跑步(间歇)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>周三
 Wed
-游泳(主)</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+🏊游泳(主课)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>周四
 Thu
-跑步(节奏)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+🏃跑步(节奏)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>周五
 Fri
-游泳(恢复)</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
+🏊游泳(恢复)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>周六
 Sat
-Brick</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+🧱Brick</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>周日
 Sun
-长骑</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="58" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+🚴长骑</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="72" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>W1
 03/10
--
+～
 03/16</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Build
 1</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>💤 REST</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>💤
+REST</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>🏃 间歇跑 5×800m
 热身10min Z2 → 5×800m Z4（间歇90s Z2）→ 放松10min Z2
@@ -688,15 +762,21 @@
 📏 约7–8km</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池技术+有氧 W1
-200m慢爬，感受水感
-❤ Z2 114–132 bpm
-📏 约1.1km</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳主课 W1｜单臂划水
+本周主题：单臂划水——感受高肘入水和掌心抓水
+热身：200m 慢爬，放松肩膀
+技术组：6×25m 单臂划水（左右各3组）
+  ▸ 一侧手臂划水，另一侧贴体或前伸
+  ▸ 重点：入水时手掌先入，手肘不能先落
+主体：6×100m Z2，间歇20s，全程保持单臂的入水感
+放松：200m 慢游
+💡 今天不追速度，只练手型
+❤ Z2 114–132 bpm | 📏 约1.1km</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>🏃 节奏跑 35min
 热身10min Z2 → 15min Z3节奏跑 → 放松10min Z2
@@ -704,23 +784,27 @@
 📏 约5–6km</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池恢复游 W1-Fri
-200m
-❤ Z2 114–132 bpm
-📏 约1.0km</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳恢复课 W1｜单臂复习
+本周主题复习：单臂划水
+热身：150m
+技术复习：4×25m 单臂划水（感受和周三的区别）
+轻松游：300m Z2 持续，把单臂的手型带入完整动作
+放松：150m
+💡 恢复课量小，重点是把技术睡一觉后再确认
+❤ Z2 114–132 bpm | 📏 约0.8km</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>🧱 Brick 骑行60min + 跑步25min
-骑行60min Z2–Z3（含15min热身/放松）→ 不休息立即换跑步25min Z3（…
+骑行60min Z2–Z3（含15min热身/放松）→ 不休息立即换跑步25min Z3（体验腿部沉重感）
 ❤ 骑行Z2–Z3 / 跑步Z3 133–150 bpm
 📏 骑行约25km + 跑步约3.5km</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I4" s="9" t="inlineStr">
         <is>
           <t>🚴 长骑 Z2 75min
 全程Z2有氧骑行，稳定心率，感受节奏
@@ -729,27 +813,28 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="5" ht="72" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>W2
 03/17
--
+～
 03/23</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Build
 1</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>💤 REST</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>💤
+REST</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>🏃 节奏跑 45min
 热身10min Z2 → 25min Z3持续节奏跑 → 放松10min Z2
@@ -757,15 +842,20 @@
 📏 约6–7km</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池技术+配速 W2
-300m慢爬
-❤ Z2–Z3 114–150 bpm
-📏 约1.4km</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳主课 W2｜单臂进阶
+本周主题：单臂——加入转体配合
+热身：200m
+技术组：6×25m 单臂划水（加入髋部转体，手入水时同侧髋下压）
+  ▸ 感受：不是手臂在划水，是身体在转动带动手臂
+主体：4×150m Z2，间歇25s
+放松：200m
+💡 本周比上周多转体，速度会快一点
+❤ Z2 114–132 bpm | 📏 约1.15km</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>🏃 轻松跑 40min Z2
 全程Z2，有氧恢复跑，感觉轻松
@@ -773,23 +863,27 @@
 📏 约5–6km</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池恢复游 W2-Fri
-200m
-❤ Z2 114–132 bpm
-📏 约1.0km</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳恢复课 W2｜单臂+转体巩固
+本周主题复习：单臂+转体
+热身：150m
+技术复习：4×25m 单臂+转体（慢速，感受髋带肩）
+轻松游：350m Z2 持续
+放松：100m
+💡 两周单臂训练到这里，入水手型应该稳定了
+❤ Z2 114–132 bpm | 📏 约0.8km</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>🧱 Brick 骑行80min + 跑步25min
-骑行80min Z2–Z3（含热身放松）→ 立即换跑步25min Z3，后10min尝试Z…
+骑行80min Z2–Z3（含热身放松）→ 立即换跑步25min Z3，后10min尝试Z4
 ❤ 骑行Z2–Z3 / 跑步Z3–Z4
 📏 骑行约33km + 跑步约3.5km</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr">
         <is>
           <t>🚴 长骑 Z2 85min
 全程Z2，后20min可升至Z3
@@ -798,27 +892,28 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>W3
 03/24
--
+～
 03/30</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Build
 1</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>💤 REST</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>💤
+REST</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>🏃 间歇跑 6×800m
 热身10min → 6×800m Z4（间歇90s）→ 放松10min
@@ -826,15 +921,21 @@
 📏 约8–9km</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池技术+阈值 W3
-300m
-❤ Z3 133–150 bpm
-📏 约1.7km</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳主课 W3｜追手/滑翔
+本周主题：追手——感受水中滑翔和减少阻力
+热身：200m
+技术组：6×25m 追手（前手等后手追上才开始划，感受身体在水中的滑翔）
+  ▸ 两手短暂相遇于头部前方
+  ▸ 感受：身体像一根细长的鱼，不是在搅水
+主体：3×200m Z2，间歇30s
+放松：200m
+💡 动作会变慢，这是正常的，感受延伸感
+❤ Z2 114–132 bpm | 📏 约1.2km</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>🏃 节奏跑 45min
 热身10min → 25min Z3节奏跑 → 放松10min
@@ -842,15 +943,19 @@
 📏 约6–7km</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池恢复游 W3-Fri
-200m
-❤ Z2 114–132 bpm
-📏 约0.9km</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳恢复课 W3｜追手巩固
+本周主题复习：追手
+热身：150m
+技术复习：4×25m 追手（放慢节奏体会滑翔停顿感）
+轻松游：300m Z2
+放松：150m
+💡 Build 1量大，周五以恢复为主
+❤ Z2 114–132 bpm | 📏 约0.8km</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>🧱 Brick 骑行90min + 跑步30min
 骑行90min → 立即跑步30min Z3–Z4（比赛节奏体验）
@@ -858,7 +963,7 @@
 📏 骑行约38km + 跑步约4.5km</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>🚴 长骑 Z2–Z3 100min
 热身15min → 70min Z2–Z3稳态 → 放松15min。Build 1最长骑行
@@ -867,26 +972,27 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>W4
 03/31
--
+～
 04/06</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Recovery</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>💤 REST</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>💤
+REST</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>🏃 轻松跑 40min Z2
 恢复周。全程Z2，不追配速，享受跑步
@@ -894,15 +1000,19 @@
 📏 约5–6km</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池技术恢复 W4
-200m
-❤ Z2 114–132 bpm
-📏 约1.0km</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳主课 W4｜追手进阶（恢复周）
+本周主题：追手——把滑翔感带入正常配速
+热身：200m
+技术组：4×25m 追手（尝试在不降速的情况下保持延伸感）
+主体：4×100m Z2，间歇20s（轻松节奏，恢复周）
+放松：200m
+💡 恢复周量减40%，不追强度
+❤ Z2 114–132 bpm | 📏 约0.9km</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>🏃 轻松跑 30min Z2
 恢复周。全程Z2，不追配速
@@ -910,15 +1020,19 @@
 📏 约4km</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池技术游 W4-Fri
-150m
-❤ Z2 114–132 bpm
-📏 约0.8km</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳恢复课 W4｜自选技术
+恢复周最轻量课
+热身：100m
+自选技术：4×25m（单臂或追手，选感觉好的那个）
+轻松游：200m Z2
+放松：100m
+💡 动一动别僵着，不要强度
+❤ Z2 114–132 bpm | 📏 约0.6km</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>🧱 轻量Brick 骑行60min + 跑步15min
 恢复周brick：骑行60min Z2 → 跑步15min Z2，维持神经肌肉感觉
@@ -926,7 +1040,7 @@
 📏 骑行约25km + 跑步约2km</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I7" s="9" t="inlineStr">
         <is>
           <t>🚴 轻松长骑 60min Z2
 恢复周。全程Z2，完全有氧，不冲强度
@@ -935,27 +1049,28 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+    <row r="8" ht="72" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>W5
 04/07
--
+～
 04/13</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Build
 2</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>💤 REST</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>💤
+REST</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>🏃 间歇跑 6×1000m
 热身10min → 6×1000m Z4（间歇2min Z2）→ 放松10min
@@ -963,15 +1078,21 @@
 📏 约9–10km</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池技术+耐力 W5
-300m
-❤ Z3 133–150 bpm
-📏 约1.5km</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳主课 W5｜双侧呼吸
+本周主题：双侧呼吸——左右均衡，消除划水不对称
+热身：200m
+技术组：6×25m 双侧呼吸（每3次划水呼吸一次，左右交替）
+  ▸ 惯用右侧的人：专门加练左侧呼吸4×25m
+  ▸ 呼吸时头不要抬，贴水面转头
+主体：6×100m Z2，间歇20s，全程双侧呼吸
+放松：200m
+💡 会很别扭，这是正常的，坚持两周
+❤ Z2 114–132 bpm | 📏 约1.2km</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>🏃 节奏跑 50min
 热身10min → 30min Z3节奏跑 → 放松10min
@@ -979,23 +1100,27 @@
 📏 约7km</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池恢复游 W5-Fri
-200m
-❤ Z2 114–132 bpm
-📏 约1.0km</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳恢复课 W5｜双侧呼吸巩固
+本周主题复习：双侧呼吸
+热身：150m
+技术复习：6×25m 双侧呼吸（刻意慢速，感受左侧呼吸）
+轻松游：350m Z2，尽量保持双侧
+放松：100m
+💡 周五只做复习，不加新东西
+❤ Z2 114–132 bpm | 📏 约0.9km</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>🧱 Brick 骑行90min + 跑步30min
-骑行90min Z2–Z3 → 立即跑步30min（前20min Z3，后10min Z4…
+骑行90min Z2–Z3 → 立即跑步30min（前20min Z3，后10min Z4尝试比赛配速）
 ❤ 骑行Z2–Z3 / 跑步Z3–Z4
 📏 骑行约38km + 跑步约4.5km</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I8" s="9" t="inlineStr">
         <is>
           <t>🚴 长骑 Z2–Z3 105min
 热身15min → 75min Z2–Z3 → 放松15min
@@ -1004,27 +1129,28 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+    <row r="9" ht="72" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>W6
 04/14
--
+～
 04/20</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Build
 2</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>💤 REST</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>💤
+REST</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>🏃 节奏跑 55min
 热身10min → 35min Z3持续（目标全程均速）→ 放松10min
@@ -1032,15 +1158,21 @@
 📏 约7–8km</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池技术+阈值 W6
-300m
-❤ Z3–Z4 133–165 bpm
-📏 约1.7km</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳主课 W6｜双侧呼吸进阶
+本周主题：双侧呼吸——提高节奏，不降速
+热身：200m
+技术组：4×25m 双侧（感受节奏稳定了吗？）
+主体：3×300m Z2–Z3，间歇40s，全程双侧呼吸
+  ▸ 第1组：3次呼一次（双侧）
+  ▸ 第2–3组：如果累可以2次呼一次（单侧）
+放松：200m
+💡 两周后双侧呼吸应该自然很多了
+❤ Z2–Z3 114–150 bpm | 📏 约1.3km</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>🏃 轻松跑 40min Z2
 全程Z2有氧恢复，为周末Brick蓄力
@@ -1048,23 +1180,27 @@
 📏 约5–6km</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池恢复游 W6-Fri
-200m
-❤ Z2 114–132 bpm
-📏 约1.0km</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳恢复课 W6｜双侧呼吸收尾
+本周主题复习：双侧呼吸最后一次
+热身：150m
+技术复习：4×25m 双侧（轻松节奏）
+轻松游：400m Z2
+放松：150m
+💡 从下周开始打腿，双侧呼吸已成习惯
+❤ Z2 114–132 bpm | 📏 约0.9km</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>🧱 Brick 骑行100min + 跑步35min
-骑行100min Z2–Z3 → 立即跑步35min（前15min Z3，中15min Z…
+骑行100min Z2–Z3 → 立即跑步35min（前15min Z3，中15min Z4，后5min放松）
 ❤ 骑行Z2–Z3 / 跑步Z3–Z4
 📏 骑行约42km + 跑步约5km</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="I9" s="9" t="inlineStr">
         <is>
           <t>🚴 长骑 Z2 110min
 全程Z2稳态。专注有氧效率
@@ -1073,27 +1209,28 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
+    <row r="10" ht="72" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>W7
 04/21
--
+～
 04/27</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Build
 2</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>💤 REST</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>💤
+REST</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>🏃 间歇跑 8×800m
 热身10min → 8×800m Z4（间歇90s）→ 放松10min
@@ -1101,15 +1238,21 @@
 📏 约10–11km</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池速度耐力 W7
-400m（含4×25m随意技术复习）
-❤ Z3–Z4 133–165 bpm
-📏 约2.0km</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳主课 W7｜打腿节奏
+本周主题：两拍腿——铁三最省力的打腿方式
+热身：200m
+技术组：
+  4×25m 夹板打腿（只用腿，感受节奏）
+  4×25m 两拍腿全划（每个划水循环踢两次腿）
+主体：4×200m Z2，间歇30s，专注两拍腿
+放松：200m
+💡 铁三不需要六拍腿，两拍省力留体力给骑跑
+❤ Z2 114–132 bpm | 📏 约1.3km</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>🏃 节奏跑 55min
 热身10min → 35min Z3节奏跑 → 放松10min
@@ -1117,23 +1260,27 @@
 📏 约7–8km</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池恢复游 W7-Fri
-200m
-❤ Z2 114–132 bpm
-📏 约1.0km</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳恢复课 W7｜打腿巩固
+Build 2峰值周，周五只维持感觉
+热身：150m
+技术复习：4×25m 两拍腿（感受轻盈）
+轻松游：400m Z2
+放松：150m
+💡 腿已经很累了，不要加强度
+❤ Z2 114–132 bpm | 📏 约0.9km</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>🧱 Brick 骑行110min + 跑步35min
-最长brick周。骑行110min Z2–Z3 → 立即跑步35min Z3–Z4（比赛模…
+最长brick周。骑行110min Z2–Z3 → 立即跑步35min Z3–Z4（比赛模拟）
 ❤ 骑行Z2–Z3 / 跑步Z3–Z4 133–165 bpm
 📏 骑行约45km + 跑步约5km</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I10" s="9" t="inlineStr">
         <is>
           <t>🚴 长骑 Z2–Z3 120min
 热身15min → 90min Z2–Z3 → 放松15min。Build 2最长骑行
@@ -1142,26 +1289,27 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="11" ht="72" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>W8
 04/28
--
+～
 05/04</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Recovery</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>💤 REST</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>💤
+REST</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>🏃 轻松跑 40min Z2
 恢复周，全程Z2，感觉非常轻松
@@ -1169,15 +1317,19 @@
 📏 约5–6km</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池技术恢复 W8
-200m
-❤ Z2 114–132 bpm
-📏 约1.0km</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳主课 W8｜打腿节奏（恢复周）
+本周主题：打腿——整合入完整动作（恢复周，量减40%）
+热身：200m
+技术组：4×25m 两拍腿（感受上下肢配合）
+主体：4×100m Z2，间歇20s
+放松：200m
+💡 恢复周，不追距离
+❤ Z2 114–132 bpm | 📏 约0.9km</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>🏃 轻松跑 35min Z2
 恢复周，全程Z2
@@ -1185,15 +1337,19 @@
 📏 约4–5km</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池激活游 W8-Fri
-150m
-❤ Z2 114–132 bpm
-📏 约0.7km</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳恢复课 W8｜自选技术最轻量
+恢复周最轻量课
+热身：100m
+自选技术：4×25m（单臂/追手/两拍腿 随意选）
+轻松游：200m Z2
+放松：100m
+💡 四周技术练习全部完成，下周开始整合配速
+❤ Z2 114–132 bpm | 📏 约0.6km</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>🧱 轻量Brick 骑行60min + 跑步20min
 恢复brick：骑行60min Z2 → 跑步20min Z2–Z3，轻松完成
@@ -1201,7 +1357,7 @@
 📏 骑行约25km + 跑步约3km</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="I11" s="9" t="inlineStr">
         <is>
           <t>🚴 轻松长骑 65min Z2
 恢复周。全程Z2，不冲强度
@@ -1210,26 +1366,27 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="58" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="12" ht="72" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>W9
 05/05
--
+～
 05/11</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Peak</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>💤 REST</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>💤
+REST</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>🏃 比赛配速跑 50min
 热身10min → 3×10min比赛配速Z4（3min Z2恢复）→ 放松10min
@@ -1237,15 +1394,21 @@
 📏 约7–8km</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>🏊 比赛模拟游泳 W9
-400m（含4×25m激活冲刺）
-❤ Z3 133–150 bpm
-📏 约1.5km（含750m比赛模拟）</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳主课 W9｜整合配速
+本周主题：把所有技术整合进比赛节奏
+热身：200m
+激活：4×25m 随选技术（感觉好的那个）
+主体：3×400m Z3，间歇45s
+  ▸ 每400m用双侧呼吸+两拍腿
+  ▸ 保持均速，不要冲前段
+放松：200m
+💡 比赛距离750m，3×400m感受一下这个强度
+❤ Z3 133–150 bpm | 📏 约1.6km</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>🏃 比赛配速跑 40min
 热身10min → 2×8min Z4比赛配速（3min Z2恢复）→ 放松10min
@@ -1253,15 +1416,18 @@
 📏 约6–7km</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池节奏游 W9-Fri
-200m
-❤ Z3 133–150 bpm
-📏 约1.0km</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳恢复课 W9｜配速感保持
+本周主题复习：整合配速
+热身：150m
+节奏组：3×100m Z3，间歇20s
+放松：200m
+💡 峰值期，周五保持感觉不加量
+❤ Z3 133–150 bpm | 📏 约0.75km</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>🧱 Brick 比赛模拟 骑行40min + 跑步25min
 缩短距离全强度：骑行40min（比赛配速Z4）→ 立即跑步25min（比赛配速Z4）
@@ -1269,7 +1435,7 @@
 📏 骑行约18km + 跑步约4km</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="I12" s="9" t="inlineStr">
         <is>
           <t>🚴 长骑 含20km比赛模拟 90min
 热身15min → 20min Z2 → 20km比赛距离全力Z4 → 放松15min
@@ -1278,26 +1444,27 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="58" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
+    <row r="13" ht="72" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>W10
 05/12
--
+～
 05/18</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Peak</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>💤 REST</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>💤
+REST</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>🏃 间歇跑 5×1000m
 热身10min → 5×1000m Z4（2min Z2恢复）→ 放松10min
@@ -1305,15 +1472,21 @@
 📏 约9–10km</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>🏊 游泳速度强化 W10
-300m
-❤ Z3–Z4 133–165 bpm
-📏 约1.6km</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳主课 W10｜比赛节奏强化
+本周主题：750m比赛全程模拟
+热身：200m
+激活：4×25m 快速（感受比赛出发节奏）
+主体：750m 持续 Z3（完整模拟比赛距离）
+  ▸ 前100m不要冲，找节奏
+  ▸ 全程双侧呼吸+两拍腿
+放松：200m
+💡 这是赛前最后一次全距离模拟
+❤ Z3 133–150 bpm | 📏 约1.35km</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>🏃 节奏跑 45min
 热身10min → 25min Z3–Z4节奏跑 → 放松10min
@@ -1321,23 +1494,25 @@
 📏 约6–7km</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池节奏游 W10-Fri
-200m
-❤ Z3 133–150 bpm
-📏 约1.0km</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳恢复课 W10｜节奏保持
+热身：150m
+节奏组：2×200m Z3，间歇30s
+放松：150m
+💡 赛前强化周，周五控制量
+❤ Z3 133–150 bpm | 📏 约0.7km</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>🧱 Brick 全距离模拟 骑行50min + 跑步20min
-最接近比赛强度：骑行50min（比赛配速）→ 立即换装 → 跑步20min（比赛配速5km…
+最接近比赛强度：骑行50min（比赛配速）→ 立即换装 → 跑步20min（比赛配速5km前4km）
 ❤ 骑行Z4 / 跑步Z4
 📏 骑行约22km + 跑步约4km</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="I13" s="9" t="inlineStr">
         <is>
           <t>🚴 长骑阈值强化 90min
 热身15min → 4×10min Z4（3min Z2恢复）→ 放松15min
@@ -1346,26 +1521,27 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="58" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
+    <row r="14" ht="72" customHeight="1">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>W11
 05/19
--
+～
 05/25</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>Taper</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>💤 REST</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>💤
+REST</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>🏃 减量跑 35min 含比赛配速
 热身10min → 3×5min比赛配速Z4（2min Z2恢复）→ 放松10min
@@ -1373,15 +1549,19 @@
 📏 约5–6km</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>🏊 减量游泳 W11
-200m
-❤ Z2–Z3 114–150 bpm
-📏 约0.9km</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳减量课 W11｜保持感觉
+减量周：量减50%，只维持水感和节奏
+热身：200m
+激活：4×25m 快速（保持高肘入水感）
+主体：4×100m Z2–Z3，间歇20s
+放松：200m
+💡 不加新技术，不追强度，感觉好就够了
+❤ Z2–Z3 114–150 bpm | 📏 约0.9km</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>🏃 减量跑 30min
 热身10min → 10min Z3（含短暂比赛配速感）→ 放松10min
@@ -1389,23 +1569,27 @@
 📏 约4km</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>🏊 泳池减量游 W11-Fri
-150m
-❤ Z2 114–132 bpm
-📏 约0.5km</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>🏊 游泳减量课 W11｜最后技术确认
+减量周最后一次游泳
+热身：100m
+技术确认：4×25m（单臂+双侧呼吸+两拍腿，各感受一遍）
+轻松游：200m Z2
+放松：100m
+💡 技术checklist：入水手型✓ 双侧呼吸✓ 两拍腿✓
+❤ Z2 114–132 bpm | 📏 约0.6km</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>🧱 最后Brick 骑行30min + 跑步15min
-最终激活。骑行30min（20min Z2 + 10min比赛配速）→ 跑步15min Z…
+最终激活。骑行30min（20min Z2 + 10min比赛配速）→ 跑步15min Z3
 ❤ 比赛配速段Z4，其余Z2–Z3
 📏 骑行约12km + 跑步约2km</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr">
+      <c r="I14" s="9" t="inlineStr">
         <is>
           <t>🚴 减量骑 50min Z2
 全程Z2，感受腿部弹性。减量周，不追强度
@@ -1414,27 +1598,28 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="58" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
+    <row r="15" ht="72" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>W12
 05/26
--
+～
 05/30</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>Race
 Week</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>💤 REST</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>💤
+REST</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>🏃 赛前激活跑 20min
 超轻松。10min Z2 + 2×1min比赛配速 + 7min Z2放松。保持腿感
@@ -1442,15 +1627,18 @@
 📏 约2.5km</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>🏊 赛前激活游泳 W12
-200m慢游
-❤ Z2–Z3
-📏 约0.6km</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>🏊 赛前激活游 W12｜只维持感觉
+比赛在周六(5/30)，今天是周三
+热身：200m 超轻松
+激活：4×25m（感受水感，不思考技术）
+放松：200m
+💡 能量储备第一，不要消耗，让肌肉记住感觉就好
+❤ Z2 114–132 bpm | 📏 约0.6km</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>🏃 赛前激活跑 15min
 超轻松。5min Z2 + 2×1min比赛配速 + 8min放松
@@ -1458,47 +1646,543 @@
 📏 约2km</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>💤 REST</t>
         </is>
       </c>
-      <c r="H14" s="13" t="inlineStr">
-        <is>
-          <t>🏆 🏆 比赛日！Sprint Triathlon
+      <c r="H15" s="15" t="inlineStr">
+        <is>
+          <t>🏆 比赛日！
+🏆 比赛日！Sprint Triathlon
 游泳750m → T1换装 → 骑行20km → T2换装 → 跑步5km
-✅ 出发策略…
-❤ 全力比赛，服从身体感觉
-📏 750m + 20km + 5km</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
+✅ 出发策略：
+• 游泳：控制节奏，不冲刺开头，Z3稳定
+• 骑行：前5km稳定进入Z3–Z4，维持均速
+• 跑步：前1km忍住腿沉，2km后加速，最后1km全力
+加油！🔥</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>💤 REST</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="14" t="inlineStr">
-        <is>
-          <t>图例：🏃跑步  🚴骑行  🏊游泳  🧱Brick(骑→跑无停顿)  🏆比赛日  💤休息  | Build 1/2: 强度积累  Recovery: 减量-40%  Peak: 比赛强度  Taper: 减量-50%</t>
+    <row r="16" ht="14" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>图例：🏃跑步  🚴骑行  🏊游泳  🧱Brick(骑→跑不停)  🏆比赛  💤休息  | 蓝=Build  绿=Recovery  黄=Build2  橙=Peak  红=Taper  紫=Race Week</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A16:I16"/>
   </mergeCells>
-  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.2" footer="0.2"/>
+  <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader>&amp;C&amp;"微软雅黑,Bold"&amp;14Zikun Sprint Triathlon 12-Week Training Plan_x000a_&amp;"微软雅黑,Regular"&amp;8Race: 2026-05-30  |  HRmax: 186 bpm  |  Z2: 114-132  Z3: 133-150  Z4: 151-165</oddHeader>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>游泳技术路线详解 · Wk1–12 每周主题</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>周次</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>主题技术</t>
+        </is>
+      </c>
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>周三主课内容</t>
+        </is>
+      </c>
+      <c r="D2" s="18" t="inlineStr">
+        <is>
+          <t>周五恢复课内容</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>W1
+Build 1</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>单臂划水</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>【游泳主课 W1｜单臂划水】
+本周主题：单臂划水——感受高肘入水和掌心抓水
+热身：200m 慢爬，放松肩膀
+技术组：6×25m 单臂划水（左右各3组）
+  ▸ 一侧手臂划水，另一侧贴体或前伸
+  ▸ 重点：入水时手掌先入，手肘不能先落
+主体：6×100m Z2，间歇20s，全程保持单臂的入水感
+放松：200m 慢游
+💡 今天不追速度，只练手型
+❤ Z2 114–132 bpm | 📏 约1.1km</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>【游泳恢复课 W1｜单臂复习】
+本周主题复习：单臂划水
+热身：150m
+技术复习：4×25m 单臂划水（感受和周三的区别）
+轻松游：300m Z2 持续，把单臂的手型带入完整动作
+放松：150m
+💡 恢复课量小，重点是把技术睡一觉后再确认
+❤ Z2 114–132 bpm | 📏 约0.8km</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>W2
+Build 1</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>单臂+转体</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>【游泳主课 W2｜单臂进阶】
+本周主题：单臂——加入转体配合
+热身：200m
+技术组：6×25m 单臂划水（加入髋部转体，手入水时同侧髋下压）
+  ▸ 感受：不是手臂在划水，是身体在转动带动手臂
+主体：4×150m Z2，间歇25s
+放松：200m
+💡 本周比上周多转体，速度会快一点
+❤ Z2 114–132 bpm | 📏 约1.15km</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>【游泳恢复课 W2｜单臂+转体巩固】
+本周主题复习：单臂+转体
+热身：150m
+技术复习：4×25m 单臂+转体（慢速，感受髋带肩）
+轻松游：350m Z2 持续
+放松：100m
+💡 两周单臂训练到这里，入水手型应该稳定了
+❤ Z2 114–132 bpm | 📏 约0.8km</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="90" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>W3
+Build 1</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>追手/滑翔</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>【游泳主课 W3｜追手/滑翔】
+本周主题：追手——感受水中滑翔和减少阻力
+热身：200m
+技术组：6×25m 追手（前手等后手追上才开始划，感受身体在水中的滑翔）
+  ▸ 两手短暂相遇于头部前方
+  ▸ 感受：身体像一根细长的鱼，不是在搅水
+主体：3×200m Z2，间歇30s
+放松：200m
+💡 动作会变慢，这是正常的，感受延伸感
+❤ Z2 114–132 bpm | 📏 约1.2km</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>【游泳恢复课 W3｜追手巩固】
+本周主题复习：追手
+热身：150m
+技术复习：4×25m 追手（放慢节奏体会滑翔停顿感）
+轻松游：300m Z2
+放松：150m
+💡 Build 1量大，周五以恢复为主
+❤ Z2 114–132 bpm | 📏 约0.8km</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>W4
+Recovery</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>追手进阶</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>【游泳主课 W4｜追手进阶（恢复周）】
+本周主题：追手——把滑翔感带入正常配速
+热身：200m
+技术组：4×25m 追手（尝试在不降速的情况下保持延伸感）
+主体：4×100m Z2，间歇20s（轻松节奏，恢复周）
+放松：200m
+💡 恢复周量减40%，不追强度
+❤ Z2 114–132 bpm | 📏 约0.9km</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>【游泳恢复课 W4｜自选技术】
+恢复周最轻量课
+热身：100m
+自选技术：4×25m（单臂或追手，选感觉好的那个）
+轻松游：200m Z2
+放松：100m
+💡 动一动别僵着，不要强度
+❤ Z2 114–132 bpm | 📏 约0.6km</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>W5
+Build 2</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>双侧呼吸</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>【游泳主课 W5｜双侧呼吸】
+本周主题：双侧呼吸——左右均衡，消除划水不对称
+热身：200m
+技术组：6×25m 双侧呼吸（每3次划水呼吸一次，左右交替）
+  ▸ 惯用右侧的人：专门加练左侧呼吸4×25m
+  ▸ 呼吸时头不要抬，贴水面转头
+主体：6×100m Z2，间歇20s，全程双侧呼吸
+放松：200m
+💡 会很别扭，这是正常的，坚持两周
+❤ Z2 114–132 bpm | 📏 约1.2km</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>【游泳恢复课 W5｜双侧呼吸巩固】
+本周主题复习：双侧呼吸
+热身：150m
+技术复习：6×25m 双侧呼吸（刻意慢速，感受左侧呼吸）
+轻松游：350m Z2，尽量保持双侧
+放松：100m
+💡 周五只做复习，不加新东西
+❤ Z2 114–132 bpm | 📏 约0.9km</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>W6
+Build 2</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>双侧呼吸进阶</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>【游泳主课 W6｜双侧呼吸进阶】
+本周主题：双侧呼吸——提高节奏，不降速
+热身：200m
+技术组：4×25m 双侧（感受节奏稳定了吗？）
+主体：3×300m Z2–Z3，间歇40s，全程双侧呼吸
+  ▸ 第1组：3次呼一次（双侧）
+  ▸ 第2–3组：如果累可以2次呼一次（单侧）
+放松：200m
+💡 两周后双侧呼吸应该自然很多了
+❤ Z2–Z3 114–150 bpm | 📏 约1.3km</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>【游泳恢复课 W6｜双侧呼吸收尾】
+本周主题复习：双侧呼吸最后一次
+热身：150m
+技术复习：4×25m 双侧（轻松节奏）
+轻松游：400m Z2
+放松：150m
+💡 从下周开始打腿，双侧呼吸已成习惯
+❤ Z2 114–132 bpm | 📏 约0.9km</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>W7
+Build 2</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>打腿节奏</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>【游泳主课 W7｜打腿节奏】
+本周主题：两拍腿——铁三最省力的打腿方式
+热身：200m
+技术组：
+  4×25m 夹板打腿（只用腿，感受节奏）
+  4×25m 两拍腿全划（每个划水循环踢两次腿）
+主体：4×200m Z2，间歇30s，专注两拍腿
+放松：200m
+💡 铁三不需要六拍腿，两拍省力留体力给骑跑
+❤ Z2 114–132 bpm | 📏 约1.3km</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>【游泳恢复课 W7｜打腿巩固】
+Build 2峰值周，周五只维持感觉
+热身：150m
+技术复习：4×25m 两拍腿（感受轻盈）
+轻松游：400m Z2
+放松：150m
+💡 腿已经很累了，不要加强度
+❤ Z2 114–132 bpm | 📏 约0.9km</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>W8
+Recovery</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>打腿整合</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>【游泳主课 W8｜打腿节奏（恢复周）】
+本周主题：打腿——整合入完整动作（恢复周，量减40%）
+热身：200m
+技术组：4×25m 两拍腿（感受上下肢配合）
+主体：4×100m Z2，间歇20s
+放松：200m
+💡 恢复周，不追距离
+❤ Z2 114–132 bpm | 📏 约0.9km</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>【游泳恢复课 W8｜自选技术最轻量】
+恢复周最轻量课
+热身：100m
+自选技术：4×25m（单臂/追手/两拍腿 随意选）
+轻松游：200m Z2
+放松：100m
+💡 四周技术练习全部完成，下周开始整合配速
+❤ Z2 114–132 bpm | 📏 约0.6km</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>W9
+Peak</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>整合配速</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>【游泳主课 W9｜整合配速】
+本周主题：把所有技术整合进比赛节奏
+热身：200m
+激活：4×25m 随选技术（感觉好的那个）
+主体：3×400m Z3，间歇45s
+  ▸ 每400m用双侧呼吸+两拍腿
+  ▸ 保持均速，不要冲前段
+放松：200m
+💡 比赛距离750m，3×400m感受一下这个强度
+❤ Z3 133–150 bpm | 📏 约1.6km</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>【游泳恢复课 W9｜配速感保持】
+本周主题复习：整合配速
+热身：150m
+节奏组：3×100m Z3，间歇20s
+放松：200m
+💡 峰值期，周五保持感觉不加量
+❤ Z3 133–150 bpm | 📏 约0.75km</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>W10
+Peak</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>比赛全程模拟</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>【游泳主课 W10｜比赛节奏强化】
+本周主题：750m比赛全程模拟
+热身：200m
+激活：4×25m 快速（感受比赛出发节奏）
+主体：750m 持续 Z3（完整模拟比赛距离）
+  ▸ 前100m不要冲，找节奏
+  ▸ 全程双侧呼吸+两拍腿
+放松：200m
+💡 这是赛前最后一次全距离模拟
+❤ Z3 133–150 bpm | 📏 约1.35km</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>【游泳恢复课 W10｜节奏保持】
+热身：150m
+节奏组：2×200m Z3，间歇30s
+放松：150m
+💡 赛前强化周，周五控制量
+❤ Z3 133–150 bpm | 📏 约0.7km</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>W11
+Taper</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>减量保感觉</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>【游泳减量课 W11｜保持感觉】
+减量周：量减50%，只维持水感和节奏
+热身：200m
+激活：4×25m 快速（保持高肘入水感）
+主体：4×100m Z2–Z3，间歇20s
+放松：200m
+💡 不加新技术，不追强度，感觉好就够了
+❤ Z2–Z3 114–150 bpm | 📏 约0.9km</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>【游泳减量课 W11｜最后技术确认】
+减量周最后一次游泳
+热身：100m
+技术确认：4×25m（单臂+双侧呼吸+两拍腿，各感受一遍）
+轻松游：200m Z2
+放松：100m
+💡 技术checklist：入水手型✓ 双侧呼吸✓ 两拍腿✓
+❤ Z2 114–132 bpm | 📏 约0.6km</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>W12
+Race Week</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>赛前激活</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>【赛前激活游 W12｜只维持感觉】
+比赛在周六(5/30)，今天是周三
+热身：200m 超轻松
+激活：4×25m（感受水感，不思考技术）
+放松：200m
+💡 能量储备第一，不要消耗，让肌肉记住感觉就好
+❤ Z2 114–132 bpm | 📏 约0.6km</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>